<commit_message>
Add bus ID to individual bus numbers
</commit_message>
<xml_diff>
--- a/Navigo.xlsx
+++ b/Navigo.xlsx
@@ -14,9 +14,9 @@
     <sheet name="Research_Notes" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Route_Master!$A$1:$U$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Stop_Master!$A$1:$F$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Bus_Schedule!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Route_Master!$A$1:$U$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Stop_Master!$A$1:$F$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Bus_Schedule!$B$1:$J$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">ETA_Logic!$A$1:$B$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Research_Notes!$A$1:$B$6</definedName>
   </definedNames>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="286">
   <si>
     <t>BUS NO.</t>
   </si>
@@ -604,6 +604,9 @@
     <t>ST061</t>
   </si>
   <si>
+    <t>BUS ID.</t>
+  </si>
+  <si>
     <t>ROUTE</t>
   </si>
   <si>
@@ -625,6 +628,9 @@
     <t>NOTE</t>
   </si>
   <si>
+    <t>B001</t>
+  </si>
+  <si>
     <t>Bajal → Statebank</t>
   </si>
   <si>
@@ -643,9 +649,15 @@
     <t>Public route references associate 9A/31A with Bajal–State Bank; exact operator timetable not verified.</t>
   </si>
   <si>
+    <t>B002</t>
+  </si>
+  <si>
     <t>Public route references associate 9B/26A with Bajal–State Bank; exact operator timetable not verified.</t>
   </si>
   <si>
+    <t>B003</t>
+  </si>
+  <si>
     <t>Statebank → Adyar</t>
   </si>
   <si>
@@ -655,6 +667,9 @@
     <t>Public references list 11A/27A State Bank–Adyar L. Jetty; exact private-bus timetable not verified.</t>
   </si>
   <si>
+    <t>B004</t>
+  </si>
+  <si>
     <t>06:10</t>
   </si>
   <si>
@@ -664,6 +679,9 @@
     <t>Second bus offset by 10 min for prototype simulation; replace with real timetable.</t>
   </si>
   <si>
+    <t>B005</t>
+  </si>
+  <si>
     <t>Statebank → Puttur</t>
   </si>
   <si>
@@ -673,12 +691,18 @@
     <t>Exact route/timetable supplied by user; schedule is a prototype assumption.</t>
   </si>
   <si>
+    <t>B006</t>
+  </si>
+  <si>
     <t>06:15</t>
   </si>
   <si>
     <t>20:15</t>
   </si>
   <si>
+    <t>B007</t>
+  </si>
+  <si>
     <t>Statebank → Talapady</t>
   </si>
   <si>
@@ -688,24 +712,36 @@
     <t>Public references associate route 42/48 with State Bank–Talapady; exact operator timetable not verified.</t>
   </si>
   <si>
+    <t>B008</t>
+  </si>
+  <si>
     <t>Statebank → Ullala</t>
   </si>
   <si>
     <t>Public references list State Bank–Ullal/Someshwar services; exact operator timetable not verified.</t>
   </si>
   <si>
+    <t>B009</t>
+  </si>
+  <si>
     <t>Statebank → Surathkal</t>
   </si>
   <si>
     <t>User-supplied route; schedule is prototype only.</t>
   </si>
   <si>
+    <t>B010</t>
+  </si>
+  <si>
     <t>Statebank → Kateel</t>
   </si>
   <si>
     <t>Public sources list State Bank–Kateel services; exact operator timetable not verified.</t>
   </si>
   <si>
+    <t>B011</t>
+  </si>
+  <si>
     <t>Local Private</t>
   </si>
   <si>
@@ -715,16 +751,25 @@
     <t>Route covers Kulshekar -&gt; Bikkarnakatta -&gt; Kadri -&gt; Jyothi -&gt; State Bank.</t>
   </si>
   <si>
+    <t>B012</t>
+  </si>
+  <si>
     <t>Kulshekar -&gt; Statebank (via Kankanady)</t>
   </si>
   <si>
     <t>Route covers Kulshekar -&gt; Bikkarnakatta -&gt; Kankanady -&gt; Falnir -&gt; State Bank.</t>
   </si>
   <si>
+    <t>B013</t>
+  </si>
+  <si>
     <t>Neermarga -&gt; Statebank (via Kulshekar)</t>
   </si>
   <si>
     <t>Route covers Kulshekar -&gt; Nanthur -&gt; Bunts Hostel -&gt; Jyothi -&gt; State Bank.</t>
+  </si>
+  <si>
+    <t>B014</t>
   </si>
   <si>
     <t>Bajpe -&gt; Statebank (via Kulshekar)</t>
@@ -865,7 +910,7 @@
     <numFmt numFmtId="180" formatCode="h:mm"/>
     <numFmt numFmtId="181" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -877,13 +922,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1354,148 +1392,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1507,10 +1545,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2782,7 +2820,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:U11" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:U15" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4051,7 +4089,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:F43" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:F62" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4062,28 +4100,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="65" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="65" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.8" spans="1:14">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="28.8" spans="1:15">
+      <c r="A1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>189</v>
@@ -4103,435 +4141,480 @@
       <c r="I1" s="1" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="2" ht="28.8" spans="1:14">
-      <c r="A2" s="2" t="s">
+      <c r="J1" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="2" ht="28.8" spans="1:15">
+      <c r="A2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H2" s="2">
+        <v>30</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="3" ht="28.8" spans="1:15">
+      <c r="A3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="G2" s="2">
-        <v>30</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="3" ht="28.8" spans="1:14">
-      <c r="A3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="G3" s="2">
+      <c r="H3" s="2">
         <v>20</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>199</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="4" ht="28.8" spans="1:14">
-      <c r="A4" s="2" t="s">
+      <c r="J3" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="4" ht="28.8" spans="1:15">
+      <c r="A4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>202</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H4" s="2">
+        <v>20</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="5" ht="28.8" spans="1:15">
+      <c r="A5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="2">
+        <v>20</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" t="s">
+        <v>213</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="H6" s="2">
+        <v>60</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" t="s">
+        <v>217</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="H7" s="2">
+        <v>60</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8" ht="28.8" spans="1:15">
+      <c r="A8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="H8" s="2">
+        <v>10</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="9" ht="28.8" spans="1:15">
+      <c r="A9" t="s">
+        <v>224</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H9" s="2">
+        <v>30</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="H10" s="2">
+        <v>30</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="11" ht="28.8" spans="1:15">
+      <c r="A11" t="s">
+        <v>230</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="H11" s="2">
+        <v>30</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" t="s">
+        <v>233</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="G4" s="2">
-        <v>20</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="5" ht="28.8" spans="1:14">
-      <c r="A5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="G5" s="2">
-        <v>20</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="G6" s="2">
-        <v>60</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="G7" s="2">
-        <v>60</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="8" ht="28.8" spans="1:14">
-      <c r="A8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="G8" s="2">
-        <v>10</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="9" ht="28.8" spans="1:14">
-      <c r="A9" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="G9" s="2">
-        <v>30</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="G10" s="2">
-        <v>30</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="11" ht="28.8" spans="1:14">
-      <c r="A11" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="G11" s="2">
-        <v>30</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E12" s="4">
+      <c r="F12" s="4">
         <v>0.25</v>
       </c>
-      <c r="F12" s="4">
+      <c r="G12" s="4">
         <v>0.854166666666667</v>
       </c>
-      <c r="G12" s="3">
+      <c r="H12" s="3">
         <v>15</v>
       </c>
-      <c r="H12" s="3" t="s">
-        <v>199</v>
-      </c>
       <c r="I12" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="J12" s="3"/>
+        <v>201</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>236</v>
+      </c>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
-    </row>
-    <row r="13" spans="1:14">
-      <c r="A13" s="3">
+      <c r="O12" s="3"/>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" t="s">
+        <v>237</v>
+      </c>
+      <c r="B13" s="3">
         <v>4</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>222</v>
-      </c>
       <c r="C13" s="3" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E13" s="4">
+        <v>238</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F13" s="4">
         <v>0.260416666666667</v>
       </c>
-      <c r="F13" s="4">
+      <c r="G13" s="4">
         <v>0.864583333333333</v>
       </c>
-      <c r="G13" s="3">
+      <c r="H13" s="3">
         <v>20</v>
       </c>
-      <c r="H13" s="3" t="s">
-        <v>199</v>
-      </c>
       <c r="I13" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="J13" s="3"/>
+        <v>201</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="3">
+      <c r="O13" s="3"/>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B14" s="3">
         <v>21</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>222</v>
-      </c>
       <c r="C14" s="3" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E14" s="4">
+        <v>241</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F14" s="4">
         <v>0.25</v>
       </c>
-      <c r="F14" s="4">
+      <c r="G14" s="4">
         <v>0.875</v>
       </c>
-      <c r="G14" s="3">
+      <c r="H14" s="3">
         <v>15</v>
       </c>
-      <c r="H14" s="3" t="s">
-        <v>199</v>
-      </c>
       <c r="I14" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="J14" s="3"/>
+        <v>201</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>242</v>
+      </c>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
-    </row>
-    <row r="15" spans="1:14">
-      <c r="A15" s="3">
+      <c r="O14" s="3"/>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15" t="s">
+        <v>243</v>
+      </c>
+      <c r="B15" s="3">
         <v>22</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>222</v>
-      </c>
       <c r="C15" s="3" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E15" s="4">
+        <v>244</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F15" s="4">
         <v>0.239583333333333</v>
       </c>
-      <c r="F15" s="4">
+      <c r="G15" s="4">
         <v>0.84375</v>
       </c>
-      <c r="G15" s="3">
+      <c r="H15" s="3">
         <v>30</v>
       </c>
-      <c r="H15" s="3" t="s">
-        <v>199</v>
-      </c>
       <c r="I15" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="J15" s="3"/>
+        <v>201</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I11" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B1:J15" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4551,114 +4634,114 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>251</v>
+        <v>266</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" ht="28.8" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -4682,50 +4765,50 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" ht="28.8" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>265</v>
+        <v>280</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>266</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>268</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>270</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>